<commit_message>
+ 500 episode with epsilon 0.4
</commit_message>
<xml_diff>
--- a/door_switch_maze/grid/DQN/episode_rewards.xlsx
+++ b/door_switch_maze/grid/DQN/episode_rewards.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B501"/>
+  <dimension ref="A1:B511"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4440,6 +4440,86 @@
         <v>0.3334375000000001</v>
       </c>
     </row>
+    <row r="502">
+      <c r="A502" t="n">
+        <v>501</v>
+      </c>
+      <c r="B502" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="n">
+        <v>502</v>
+      </c>
+      <c r="B503" t="n">
+        <v>0.881875</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="n">
+        <v>503</v>
+      </c>
+      <c r="B504" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="n">
+        <v>504</v>
+      </c>
+      <c r="B505" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="n">
+        <v>505</v>
+      </c>
+      <c r="B506" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="n">
+        <v>506</v>
+      </c>
+      <c r="B507" t="n">
+        <v>0.74125</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="n">
+        <v>507</v>
+      </c>
+      <c r="B508" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="n">
+        <v>508</v>
+      </c>
+      <c r="B509" t="n">
+        <v>0.3629687500000001</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="n">
+        <v>509</v>
+      </c>
+      <c r="B510" t="n">
+        <v>0.80453125</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="n">
+        <v>510</v>
+      </c>
+      <c r="B511" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>